<commit_message>
Release 0.8.1: integrate Neon Gothic art, directional animation and combat polish
</commit_message>
<xml_diff>
--- a/outputs/01a073ab-e45b-7f41-9fda-1b7538ae0af7/Баланс Skeleton Defender.xlsx
+++ b/outputs/01a073ab-e45b-7f41-9fda-1b7538ae0af7/Баланс Skeleton Defender.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Обзор" sheetId="1" r:id="R42c783c486d542e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Герои" sheetId="2" r:id="Rf51fc5539bd94e8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Враги" sheetId="3" r:id="Rfdb6a6534c834cf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Волны" sheetId="4" r:id="Rfa3a2fdb6bfd43c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Выход врагов" sheetId="5" r:id="R7abcd48d9cee467a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Башни" sheetId="6" r:id="Rafbaa416fd704338"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Добыча" sheetId="7" r:id="Rdfb905296e234787"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Экипировка" sheetId="8" r:id="Rcb5f51a8fe284eaa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Навыки" sheetId="9" r:id="R31076873ade4426b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Артефакты" sheetId="10" r:id="R4b06c59764df454f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Обзор" sheetId="1" r:id="R91777014302f4357"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Герои" sheetId="2" r:id="R77610574cb3c4b1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Враги" sheetId="3" r:id="R70efcf974a404abb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Волны" sheetId="4" r:id="R674229871a9b4e09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Выход врагов" sheetId="5" r:id="R4286ecddcbdb4395"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Башни" sheetId="6" r:id="Re9574001c9a74c58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Добыча" sheetId="7" r:id="Rf70376a3120e4b90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Экипировка" sheetId="8" r:id="R2cdf92b85a7a4b80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Навыки" sheetId="9" r:id="R7e3e0b67fc284efd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Артефакты" sheetId="10" r:id="R2abe9155e0d94d12"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -103,7 +103,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="33">
+  <x:fills count="42">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -265,6 +265,51 @@
         <x:fgColor rgb="FFECF5F1"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE5EEEA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFECF5F1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE5EEEA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFECF5F1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE5EEEA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFECF5F1"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="7">
     <x:border/>
@@ -305,7 +350,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="262">
+  <x:cellXfs count="285">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1027,6 +1072,73 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="211" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="8" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="8" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="8" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="8" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="8" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="8" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="8" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="8" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="8" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1248,7 +1360,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R54214aba23f24d2b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6ebd38625ba74e35"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2321,7 +2433,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6aa7437d73f845bd"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9abe19f959a44857"/>
 </x:worksheet>
 </file>
 
@@ -6773,7 +6885,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R456da1dbdda44587"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67ba7d6db5fc4963"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10373,7 +10485,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R314fef55ef4c4543"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R513126c11c2546b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10425,7 +10537,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>Версия 0.6.1: урон всех уровней повышен на 5%. Интервалы прежние; DPS указан без брони и эффектов.</x:v>
+        <x:v>Версия 0.8.1: III уровень — два эльфа. В C указан урон каждой стрелы; E учитывает обоих. Интервалы прежние.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -10457,13 +10569,13 @@
         <x:v>Уровень</x:v>
       </x:c>
       <x:c r="C5" s="15" t="str">
-        <x:v>Урон</x:v>
+        <x:v>Урон снаряда</x:v>
       </x:c>
       <x:c r="D5" s="15" t="str">
         <x:v>Интервал, с</x:v>
       </x:c>
       <x:c r="E5" s="15" t="str">
-        <x:v>DPS</x:v>
+        <x:v>DPS башни</x:v>
       </x:c>
       <x:c r="F5" s="15" t="str">
         <x:v>Радиус</x:v>
@@ -10497,7 +10609,7 @@
         <x:v>0.62</x:v>
       </x:c>
       <x:c r="E6" s="24" t="n">
-        <x:f>C6/D6</x:f>
+        <x:f>C6/D6*B43</x:f>
         <x:v>6.589601008064516</x:v>
       </x:c>
       <x:c r="F6" s="37" t="n">
@@ -10517,7 +10629,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="J6" s="29" t="str">
-        <x:v>Одна цель</x:v>
+        <x:v>Один эльф</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="39" customHeight="1">
@@ -10536,7 +10648,7 @@
         <x:v>0.5688073394495412</x:v>
       </x:c>
       <x:c r="E7" s="24" t="n">
-        <x:f>C7/D7</x:f>
+        <x:f>C7/D7*B44</x:f>
         <x:v>12.928797177822583</x:v>
       </x:c>
       <x:c r="F7" s="37" t="n">
@@ -10556,7 +10668,7 @@
         <x:v>122</x:v>
       </x:c>
       <x:c r="J7" s="31" t="str">
-        <x:v>Одна цель</x:v>
+        <x:v>Один эльф</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="39" customHeight="1">
@@ -10575,8 +10687,8 @@
         <x:v>0.5254237288135594</x:v>
       </x:c>
       <x:c r="E8" s="24" t="n">
-        <x:f>C8/D8</x:f>
-        <x:v>20.216895892741935</x:v>
+        <x:f>C8/D8*B45</x:f>
+        <x:v>40.43379178548387</x:v>
       </x:c>
       <x:c r="F8" s="37" t="n">
         <x:f>$E$20+B8*$F$20</x:f>
@@ -10595,7 +10707,7 @@
         <x:v>220</x:v>
       </x:c>
       <x:c r="J8" s="29" t="str">
-        <x:v>Одна цель</x:v>
+        <x:v>Два эльфа, две стрелы</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="39" customHeight="1">
@@ -10605,7 +10717,7 @@
       <x:c r="B9" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C9" s="169" t="n">
+      <x:c r="C9" s="167" t="n">
         <x:f>$C$21*(1+(B9-1)*$D$21)</x:f>
         <x:v>3.14076858046875</x:v>
       </x:c>
@@ -10645,7 +10757,7 @@
       <x:c r="B10" s="18" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C10" s="169" t="n">
+      <x:c r="C10" s="167" t="n">
         <x:f>$C$21*(1+(B10-1)*$D$21)</x:f>
         <x:v>5.65338344484375</x:v>
       </x:c>
@@ -10685,7 +10797,7 @@
       <x:c r="B11" s="20" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C11" s="169" t="n">
+      <x:c r="C11" s="167" t="n">
         <x:f>$C$21*(1+(B11-1)*$D$21)</x:f>
         <x:v>8.16599830921875</x:v>
       </x:c>
@@ -10725,7 +10837,7 @@
       <x:c r="B12" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C12" s="24" t="n">
+      <x:c r="C12" s="167" t="n">
         <x:f>$C$22*(1+(B12-1)*$D$22)</x:f>
         <x:v>2.1847875</x:v>
       </x:c>
@@ -10765,7 +10877,7 @@
       <x:c r="B13" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C13" s="24" t="n">
+      <x:c r="C13" s="167" t="n">
         <x:f>$C$22*(1+(B13-1)*$D$22)</x:f>
         <x:v>3.9326175</x:v>
       </x:c>
@@ -10805,7 +10917,7 @@
       <x:c r="B14" s="18" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C14" s="24" t="n">
+      <x:c r="C14" s="167" t="n">
         <x:f>$C$22*(1+(B14-1)*$D$22)</x:f>
         <x:v>5.6804475000000005</x:v>
       </x:c>
@@ -11288,7 +11400,40 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="125" t="str">
-        <x:v>Стрелы и огненные шары наносят урон после попадания. Заморозка ледяной башни действует непосредственно на цель.</x:v>
+        <x:v>Эльф готовит лук 0,20 с; интервал идёт от начала атаки. Стрелы III выпускаются из двух отдельных луков.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="27" customHeight="1">
+      <x:c r="A43" s="54" t="str">
+        <x:v>Стрелковая I</x:v>
+      </x:c>
+      <x:c r="B43" s="284" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C43" s="54" t="str">
+        <x:v>стрел/залп</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="27" customHeight="1">
+      <x:c r="A44" s="54" t="str">
+        <x:v>Стрелковая II</x:v>
+      </x:c>
+      <x:c r="B44" s="284" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C44" s="54" t="str">
+        <x:v>стрел/залп</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="27" customHeight="1">
+      <x:c r="A45" s="54" t="str">
+        <x:v>Стрелковая III</x:v>
+      </x:c>
+      <x:c r="B45" s="284" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C45" s="54" t="str">
+        <x:v>стрел/залп</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14924,11 +15069,11 @@
       <x:c r="F6" s="25" t="n">
         <x:v>300</x:v>
       </x:c>
-      <x:c r="G6" s="25" t="n">
-        <x:v>3</x:v>
+      <x:c r="G6" s="162" t="n">
+        <x:v>17.142857142857</x:v>
       </x:c>
       <x:c r="H6" s="199" t="str">
-        <x:v>Два оленя бегут сквозь врагов. Каждый поражает цель один раз и замедляет её.</x:v>
+        <x:v>От замка по всей дороге к входу за 17,143 с. Каждый олень: 10 урона один раз, отталкивание 12 ед. и замедление 50% на 3 с.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="68" customHeight="1">
@@ -14951,10 +15096,10 @@
         <x:v>300</x:v>
       </x:c>
       <x:c r="G7" s="25" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H7" s="200" t="str">
-        <x:v>Магический урон всем находящимся на карте врагам.</x:v>
+        <x:v>Всего 10 магического урона за 3 с: 4 удара по 2,5 каждые 0,75 с. Цели фиксируются при нажатии.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="68" customHeight="1">
@@ -15002,11 +15147,12 @@
       <x:c r="F9" s="25" t="n">
         <x:v>480</x:v>
       </x:c>
-      <x:c r="G9" s="25" t="n">
-        <x:v>0</x:v>
+      <x:c r="G9" s="162" t="n">
+        <x:f>B37</x:f>
+        <x:v>0.9285714285714287</x:v>
       </x:c>
       <x:c r="H9" s="200" t="str">
-        <x:v>Физический урон и замедление врагов, бывших на карте при нажатии.</x:v>
+        <x:v>Темп 70%: выпуск через 1,686 с, попадание через 2,614 с от нажатия. В G — полёт после выпуска. Замедление 50% на 5 с.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
@@ -15021,7 +15167,7 @@
     </x:row>
     <x:row r="11" ht="26" customHeight="1">
       <x:c r="A11" s="32" t="str">
-        <x:v>Для оленей урон указан за одно попадание каждого оленя. У стрелы Ахилла число поражённых целей зависит от состава карты.</x:v>
+        <x:v>Олени: урон каждого за один контакт. Гроза: суммарно за 4 удара. Стрела Ахилла: исходный список целей.</x:v>
       </x:c>
       <x:c r="B11" s="2"/>
       <x:c r="C11" s="2"/>
@@ -15105,7 +15251,7 @@
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="200" t="str">
-        <x:v>Олени: длительность</x:v>
+        <x:v>Замедление оленей</x:v>
       </x:c>
       <x:c r="B16" s="185" t="n">
         <x:v>3</x:v>
@@ -15299,7 +15445,7 @@
     </x:row>
     <x:row r="29" ht="26" customHeight="1">
       <x:c r="A29" s="32" t="str">
-        <x:v>Источник: уточнения пользователя для версии 0.6.1. Радиусы и время полёта — текущие параметры для баланса.</x:v>
+        <x:v>Источник: правила 0.8.1, balance.json и события AnimationPack. Числа таблицы не записываются в игру.</x:v>
       </x:c>
       <x:c r="B29" s="2"/>
       <x:c r="C29" s="2"/>
@@ -15319,86 +15465,159 @@
       <x:c r="G30" s="2"/>
       <x:c r="H30" s="2"/>
     </x:row>
-    <x:row r="31" ht="24" customHeight="1">
-      <x:c r="A31" s="2"/>
-      <x:c r="B31" s="2"/>
-      <x:c r="C31" s="2"/>
+    <x:row r="31" ht="27" customHeight="1">
+      <x:c r="A31" s="281" t="str">
+        <x:v>Параметры 0.8.1</x:v>
+      </x:c>
+      <x:c r="B31" s="282" t="str">
+        <x:v>Значение</x:v>
+      </x:c>
+      <x:c r="C31" s="281" t="str">
+        <x:v>Единица</x:v>
+      </x:c>
       <x:c r="D31" s="2"/>
       <x:c r="E31" s="2"/>
       <x:c r="F31" s="2"/>
       <x:c r="G31" s="2"/>
       <x:c r="H31" s="2"/>
     </x:row>
-    <x:row r="32" ht="24" customHeight="1">
-      <x:c r="A32" s="2"/>
-      <x:c r="B32" s="2"/>
-      <x:c r="C32" s="2"/>
+    <x:row r="32" ht="40" customHeight="1">
+      <x:c r="A32" s="279" t="str">
+        <x:v>E Ахилла: скорость</x:v>
+      </x:c>
+      <x:c r="B32" s="280" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="C32" s="54" t="str">
+        <x:v>×</x:v>
+      </x:c>
       <x:c r="D32" s="2"/>
       <x:c r="E32" s="2"/>
       <x:c r="F32" s="2"/>
       <x:c r="G32" s="2"/>
       <x:c r="H32" s="2"/>
     </x:row>
-    <x:row r="33" ht="24" customHeight="1">
-      <x:c r="A33" s="2"/>
-      <x:c r="B33" s="2"/>
-      <x:c r="C33" s="2"/>
+    <x:row r="33" ht="40" customHeight="1">
+      <x:c r="A33" s="279" t="str">
+        <x:v>E: исходный полёт</x:v>
+      </x:c>
+      <x:c r="B33" s="280" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="C33" s="54" t="str">
+        <x:v>с</x:v>
+      </x:c>
       <x:c r="D33" s="2"/>
       <x:c r="E33" s="2"/>
       <x:c r="F33" s="2"/>
       <x:c r="G33" s="2"/>
       <x:c r="H33" s="2"/>
     </x:row>
-    <x:row r="34" ht="24" customHeight="1">
-      <x:c r="A34" s="2"/>
-      <x:c r="B34" s="2"/>
-      <x:c r="C34" s="2"/>
+    <x:row r="34" ht="40" customHeight="1">
+      <x:c r="A34" s="279" t="str">
+        <x:v>E: исходный выпуск</x:v>
+      </x:c>
+      <x:c r="B34" s="280" t="n">
+        <x:v>1.18</x:v>
+      </x:c>
+      <x:c r="C34" s="54" t="str">
+        <x:v>с</x:v>
+      </x:c>
       <x:c r="D34" s="2"/>
       <x:c r="E34" s="2"/>
       <x:c r="F34" s="2"/>
       <x:c r="G34" s="2"/>
       <x:c r="H34" s="2"/>
     </x:row>
-    <x:row r="35" ht="24" customHeight="1">
-      <x:c r="A35" s="2"/>
-      <x:c r="B35" s="2"/>
-      <x:c r="C35" s="2"/>
+    <x:row r="35" ht="40" customHeight="1">
+      <x:c r="A35" s="279" t="str">
+        <x:v>E: исходный подъём</x:v>
+      </x:c>
+      <x:c r="B35" s="280" t="n">
+        <x:v>0.45</x:v>
+      </x:c>
+      <x:c r="C35" s="54" t="str">
+        <x:v>с</x:v>
+      </x:c>
       <x:c r="D35" s="2"/>
       <x:c r="E35" s="2"/>
       <x:c r="F35" s="2"/>
       <x:c r="G35" s="2"/>
       <x:c r="H35" s="2"/>
     </x:row>
-    <x:row r="36" ht="24" customHeight="1">
-      <x:c r="A36" s="2"/>
-      <x:c r="B36" s="2"/>
-      <x:c r="C36" s="2"/>
+    <x:row r="36" ht="40" customHeight="1">
+      <x:c r="A36" s="279" t="str">
+        <x:v>E: подъём в игре</x:v>
+      </x:c>
+      <x:c r="B36" s="283" t="n">
+        <x:f>B35/B32</x:f>
+        <x:v>0.6428571428571429</x:v>
+      </x:c>
+      <x:c r="C36" s="54" t="str">
+        <x:v>с</x:v>
+      </x:c>
       <x:c r="D36" s="2"/>
       <x:c r="E36" s="2"/>
       <x:c r="F36" s="2"/>
       <x:c r="G36" s="2"/>
       <x:c r="H36" s="2"/>
     </x:row>
-    <x:row r="37" ht="24" customHeight="1">
-      <x:c r="A37" s="2"/>
-      <x:c r="B37" s="2"/>
-      <x:c r="C37" s="2"/>
+    <x:row r="37" ht="40" customHeight="1">
+      <x:c r="A37" s="279" t="str">
+        <x:v>E: полёт в игре</x:v>
+      </x:c>
+      <x:c r="B37" s="283" t="n">
+        <x:f>B33/B32</x:f>
+        <x:v>0.9285714285714287</x:v>
+      </x:c>
+      <x:c r="C37" s="54" t="str">
+        <x:v>с</x:v>
+      </x:c>
       <x:c r="D37" s="2"/>
       <x:c r="E37" s="2"/>
       <x:c r="F37" s="2"/>
       <x:c r="G37" s="2"/>
       <x:c r="H37" s="2"/>
     </x:row>
-    <x:row r="38" ht="24" customHeight="1">
-      <x:c r="A38" s="2"/>
-      <x:c r="B38" s="2"/>
-      <x:c r="C38" s="2"/>
+    <x:row r="38" ht="40" customHeight="1">
+      <x:c r="A38" s="279" t="str">
+        <x:v>E: до попадания</x:v>
+      </x:c>
+      <x:c r="B38" s="283" t="n">
+        <x:f>(B34+B33)/B32</x:f>
+        <x:v>2.6142857142857148</x:v>
+      </x:c>
+      <x:c r="C38" s="54" t="str">
+        <x:v>с</x:v>
+      </x:c>
       <x:c r="D38" s="2"/>
       <x:c r="E38" s="2"/>
       <x:c r="F38" s="2"/>
       <x:c r="G38" s="2"/>
       <x:c r="H38" s="2"/>
     </x:row>
+    <x:row r="39" ht="40" customHeight="1">
+      <x:c r="A39" s="279" t="str">
+        <x:v>Олень: отталкивание</x:v>
+      </x:c>
+      <x:c r="B39" s="284" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C39" s="54" t="str">
+        <x:v>ед.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="40" customHeight="1">
+      <x:c r="A40" s="279" t="str">
+        <x:v>Гроза: ударов</x:v>
+      </x:c>
+      <x:c r="B40" s="284" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C40" s="54" t="str">
+        <x:v>шт.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>